<commit_message>
gitignore pra arquivos temporarios do excel + tabela atualizada
</commit_message>
<xml_diff>
--- a/Close Care/(excel) Ordem de prioridade.xlsx
+++ b/Close Care/(excel) Ordem de prioridade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\CloseCare-GEST.PROJ.SOFT\Close Care\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2E1916-E9C9-45D6-AB3D-74696C3575F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1452133-89E4-45A0-AA2D-7F712CA0EBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B4B4DFAF-313B-4775-A4C5-2B6A73696C89}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
@@ -95,10 +95,6 @@
     <t>HU13</t>
   </si>
   <si>
-    <t>Como paciente com mobilidade reduzida ou idoso, quero agendar uma consulta domiciliar selecionando o tipo de profissional, a data, o horário e 
-o meu endereço cadastrado para receber atendimento médico em casa com conforto, sem a necessidade de deslocamento.</t>
-  </si>
-  <si>
     <t>Como paciente ou profissional de saúde, quero visualizar a lista de consultas cadastradas para acompanhar os atendimentos agendados.</t>
   </si>
   <si>
@@ -181,6 +177,12 @@
   </si>
   <si>
     <t>Como paciente ou profissional de saúde, quero remarcar a data e/ou horário de um exame domiciliar já agendado por conta de imprevistos de agenda de uma ou ambas as partes.</t>
+  </si>
+  <si>
+    <t>Como paciente com mobilidade reduzida ou idoso, quero agendar uma consulta domiciliar selecionando o tipo de profissional, a data, o horário e o meu endereço cadastrado para receber atendimento médico em casa com conforto, sem a necessidade de deslocamento.</t>
+  </si>
+  <si>
+    <t>Como paciente com mobilidade reduzida ou idoso, quero agendar um exame selecionando o tipo de profissional, a data, o horário e o meu endereço cadastrado para receber atendimento médico em casa com conforto, sem a necessidade de deslocamento.</t>
   </si>
 </sst>
 </file>
@@ -803,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D1F92C-1AF3-4A95-B439-F4557C2C0F00}">
-  <dimension ref="B1:E28"/>
+  <dimension ref="B1:E30"/>
   <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
@@ -834,10 +836,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>15</v>
@@ -848,10 +850,10 @@
         <v>2</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>15</v>
@@ -862,10 +864,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>15</v>
@@ -879,7 +881,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
@@ -893,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>15</v>
@@ -907,7 +909,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>15</v>
@@ -921,7 +923,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>15</v>
@@ -935,7 +937,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>15</v>
@@ -949,7 +951,7 @@
         <v>9</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>15</v>
@@ -963,7 +965,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>15</v>
@@ -977,7 +979,7 @@
         <v>17</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>15</v>
@@ -991,7 +993,7 @@
         <v>18</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>15</v>
@@ -1002,10 +1004,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>15</v>
@@ -1016,10 +1018,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>15</v>
@@ -1033,7 +1035,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>16</v>
@@ -1047,7 +1049,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>16</v>
@@ -1061,7 +1063,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>16</v>
@@ -1072,10 +1074,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>16</v>
@@ -1086,10 +1088,10 @@
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>16</v>
@@ -1097,29 +1099,40 @@
     </row>
     <row r="26" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="B28" s="1">
+    <row r="27" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="C27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+      <c r="B30" s="1">
         <v>7</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E28" s="4" t="s">
+      <c r="D30" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ordem de prioridade recontabilizada
</commit_message>
<xml_diff>
--- a/Close Care/(excel) Ordem de prioridade.xlsx
+++ b/Close Care/(excel) Ordem de prioridade.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\GitHub\CloseCare-GEST.PROJ.SOFT\Close Care\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luism\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1452133-89E4-45A0-AA2D-7F712CA0EBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43FD511-87DF-40A6-A1F9-A76B76BF704E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B4B4DFAF-313B-4775-A4C5-2B6A73696C89}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4B4DFAF-313B-4775-A4C5-2B6A73696C89}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="47">
   <si>
     <t>ID</t>
   </si>
@@ -138,12 +138,6 @@
   </si>
   <si>
     <t>HU18</t>
-  </si>
-  <si>
-    <t>HU19</t>
-  </si>
-  <si>
-    <t>HU20</t>
   </si>
   <si>
     <t>Como paciente com falta de mobilidade ou profissional, quero cadastrar uma conta no aplicativo inserindo meus dados para acessar os serviços de atendimento domiciliar conforme o meu tipo de conta.</t>
@@ -358,7 +352,6 @@
   <dxfs count="7">
     <dxf>
       <font>
-        <b/>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -386,6 +379,22 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -447,21 +456,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -476,13 +470,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}" name="Tabela1" displayName="Tabela1" ref="B2:E21" headerRowDxfId="5" dataDxfId="3" totalsRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}" name="Tabela1" displayName="Tabela1" ref="B2:E21" headerRowDxfId="6" dataDxfId="5" totalsRowDxfId="4">
   <autoFilter ref="B2:E21" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{985DA469-90E4-4E24-8BE5-72DD8AC4D4B7}" name="Prioridade" totalsRowLabel="Total" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{8CF543ED-69A6-4089-B1C8-916B531B30CB}" name="ID" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{985DA469-90E4-4E24-8BE5-72DD8AC4D4B7}" name="Prioridade" totalsRowLabel="Total" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{8CF543ED-69A6-4089-B1C8-916B531B30CB}" name="ID" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{DF14E0CF-8CC5-458E-9DBC-9D271FF5D8AF}" name="Historia" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{E588BD5A-7EF6-439C-8B85-7F5F2AAF23CB}" name="MosCow" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{E588BD5A-7EF6-439C-8B85-7F5F2AAF23CB}" name="MosCow" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -806,18 +800,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D1F92C-1AF3-4A95-B439-F4557C2C0F00}">
   <dimension ref="B1:E30"/>
-  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="159.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="4.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="159.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="13.8" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:5" ht="14.25" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:5" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>13</v>
       </c>
@@ -831,49 +825,49 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>36</v>
-      </c>
       <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>2</v>
       </c>
       <c r="C4" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>37</v>
-      </c>
       <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>3</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>4</v>
       </c>
@@ -881,13 +875,13 @@
         <v>2</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>5</v>
       </c>
@@ -901,7 +895,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>6</v>
       </c>
@@ -915,12 +909,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>7</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>29</v>
@@ -929,12 +923,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>8</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>30</v>
@@ -943,12 +937,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>9</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>31</v>
@@ -957,12 +951,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>10</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>32</v>
@@ -971,12 +965,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <v>11</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>19</v>
@@ -985,49 +979,49 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B14" s="1">
         <v>12</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B15" s="1">
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B16" s="1">
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <v>15</v>
       </c>
@@ -1041,63 +1035,63 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <v>16</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B19" s="1">
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B20" s="1">
         <v>18</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B21" s="1">
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>24</v>
       </c>
@@ -1105,24 +1099,24 @@
         <v>2</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="C27" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B30" s="1">
         <v>7</v>
       </c>

</xml_diff>